<commit_message>
Audit HMDA filtered dimension parity
</commit_message>
<xml_diff>
--- a/apps/excel/templates/CreditAtlas-HMDA-Browser-Release-Audit-2018-2025.xlsx
+++ b/apps/excel/templates/CreditAtlas-HMDA-Browser-Release-Audit-2018-2025.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Browser selected" sheetId="1" r:id="Raf1b4600a5d44a81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App One-Year" sheetId="2" r:id="Rad94a8db599f44b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vintage deltas" sheetId="3" r:id="R4d850143c48b43fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lineage" sheetId="4" r:id="R34abd30a8df342dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method &amp; sources" sheetId="5" r:id="Rd148e2d81cc4455e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Browser selected" sheetId="1" r:id="Re5f2c24140564ba5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App One-Year" sheetId="2" r:id="Ra40549d9b13b435a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vintage deltas" sheetId="3" r:id="Rf103529d0f314adc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dimension parity" sheetId="4" r:id="Rd0ddb561d3ca46ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lineage" sheetId="5" r:id="R58fb6add88fb4e67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method &amp; sources" sheetId="6" r:id="R9a99abe7817e428b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -200,7 +201,30 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="HmdaReleaseApiLineage" displayName="HmdaReleaseApiLineage" ref="A4:G12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="HmdaFilteredDimensionApiParity" displayName="HmdaFilteredDimensionApiParity" ref="A4:O9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="15">
+    <x:tableColumn id="1" name="Scope"/>
+    <x:tableColumn id="2" name="Official filter"/>
+    <x:tableColumn id="3" name="API rows 1–8"/>
+    <x:tableColumn id="4" name="Local rows 1–8"/>
+    <x:tableColumn id="5" name="API decisions 1+2+3"/>
+    <x:tableColumn id="6" name="Local decisions 1+2+3"/>
+    <x:tableColumn id="7" name="API denied · 3"/>
+    <x:tableColumn id="8" name="Local denied · 3"/>
+    <x:tableColumn id="9" name="API denied share"/>
+    <x:tableColumn id="10" name="Local denied share"/>
+    <x:tableColumn id="11" name="Δ share · pp"/>
+    <x:tableColumn id="12" name="Local raw match"/>
+    <x:tableColumn id="13" name="API filter echo"/>
+    <x:tableColumn id="14" name="App marginal match"/>
+    <x:tableColumn id="15" name="Check"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="HmdaReleaseApiLineage" displayName="HmdaReleaseApiLineage" ref="A4:G12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Activity year"/>
     <x:tableColumn id="2" name="Browser product"/>
@@ -214,8 +238,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="HmdaAuditMethodNotes" displayName="HmdaAuditMethodNotes" ref="A3:D17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="HmdaAuditMethodNotes" displayName="HmdaAuditMethodNotes" ref="A3:D18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Item"/>
     <x:tableColumn id="2" name="Definition / value"/>
@@ -1094,7 +1118,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c1f840f09fd46da"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a6dbaa99e70428e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1708,7 +1732,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79e670a80de24d12"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re89fe6e681e44e8e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2354,12 +2378,592 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdacda774264b4a27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ad22e8bbef94eb5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="52" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="15" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="15" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="17" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="17" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="17" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="14" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="17" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="14" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>Filtered dimension parity · official 2025 Snapshot API vs local source</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+      <x:c r="F1" s="4"/>
+      <x:c r="G1" s="4"/>
+      <x:c r="H1" s="4"/>
+      <x:c r="I1" s="4"/>
+      <x:c r="J1" s="4"/>
+      <x:c r="K1" s="4"/>
+      <x:c r="L1" s="4"/>
+      <x:c r="M1" s="4"/>
+      <x:c r="N1" s="4"/>
+      <x:c r="O1" s="4"/>
+    </x:row>
+    <x:row r="2" ht="54" customHeight="1">
+      <x:c r="A2" s="7" t="str">
+        <x:v>Five spot-check scopes compared on action codes 1–8. Four marginal scopes also match the receipt-verified app report; California × product is raw/API validated but not an app intersection. Share columns are Excel formulas.</x:v>
+      </x:c>
+      <x:c r="B2" s="7"/>
+      <x:c r="C2" s="7"/>
+      <x:c r="D2" s="7"/>
+      <x:c r="E2" s="7"/>
+      <x:c r="F2" s="7"/>
+      <x:c r="G2" s="7"/>
+      <x:c r="H2" s="7"/>
+      <x:c r="I2" s="7"/>
+      <x:c r="J2" s="7"/>
+      <x:c r="K2" s="7"/>
+      <x:c r="L2" s="7"/>
+      <x:c r="M2" s="7"/>
+      <x:c r="N2" s="7"/>
+      <x:c r="O2" s="7"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="2"/>
+      <x:c r="B3" s="2"/>
+      <x:c r="C3" s="2"/>
+      <x:c r="D3" s="2"/>
+      <x:c r="E3" s="2"/>
+      <x:c r="F3" s="2"/>
+      <x:c r="G3" s="2"/>
+      <x:c r="H3" s="2"/>
+      <x:c r="I3" s="2"/>
+      <x:c r="J3" s="2"/>
+      <x:c r="K3" s="2"/>
+      <x:c r="L3" s="2"/>
+      <x:c r="M3" s="2"/>
+      <x:c r="N3" s="2"/>
+      <x:c r="O3" s="2"/>
+    </x:row>
+    <x:row r="4" ht="38" customHeight="1">
+      <x:c r="A4" s="10" t="str">
+        <x:v>Scope</x:v>
+      </x:c>
+      <x:c r="B4" s="10" t="str">
+        <x:v>Official filter</x:v>
+      </x:c>
+      <x:c r="C4" s="10" t="str">
+        <x:v>API rows 1–8</x:v>
+      </x:c>
+      <x:c r="D4" s="10" t="str">
+        <x:v>Local rows 1–8</x:v>
+      </x:c>
+      <x:c r="E4" s="10" t="str">
+        <x:v>API decisions 1+2+3</x:v>
+      </x:c>
+      <x:c r="F4" s="10" t="str">
+        <x:v>Local decisions 1+2+3</x:v>
+      </x:c>
+      <x:c r="G4" s="10" t="str">
+        <x:v>API denied · 3</x:v>
+      </x:c>
+      <x:c r="H4" s="10" t="str">
+        <x:v>Local denied · 3</x:v>
+      </x:c>
+      <x:c r="I4" s="10" t="str">
+        <x:v>API denied share</x:v>
+      </x:c>
+      <x:c r="J4" s="10" t="str">
+        <x:v>Local denied share</x:v>
+      </x:c>
+      <x:c r="K4" s="10" t="str">
+        <x:v>Δ share · pp</x:v>
+      </x:c>
+      <x:c r="L4" s="10" t="str">
+        <x:v>Local raw match</x:v>
+      </x:c>
+      <x:c r="M4" s="10" t="str">
+        <x:v>API filter echo</x:v>
+      </x:c>
+      <x:c r="N4" s="10" t="str">
+        <x:v>App marginal match</x:v>
+      </x:c>
+      <x:c r="O4" s="10" t="str">
+        <x:v>Check</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="34" customHeight="1">
+      <x:c r="A5" s="2" t="str">
+        <x:v>California state</x:v>
+      </x:c>
+      <x:c r="B5" s="2" t="str">
+        <x:v>state=CA</x:v>
+      </x:c>
+      <x:c r="C5" s="11" t="n">
+        <x:v>1161292</x:v>
+      </x:c>
+      <x:c r="D5" s="11" t="n">
+        <x:v>1161292</x:v>
+      </x:c>
+      <x:c r="E5" s="11" t="n">
+        <x:v>791639</x:v>
+      </x:c>
+      <x:c r="F5" s="11" t="n">
+        <x:v>791639</x:v>
+      </x:c>
+      <x:c r="G5" s="11" t="n">
+        <x:v>177363</x:v>
+      </x:c>
+      <x:c r="H5" s="11" t="n">
+        <x:v>177363</x:v>
+      </x:c>
+      <x:c r="I5" s="12" t="n">
+        <x:f>IFERROR(G5/E5,0)</x:f>
+        <x:v>0.2240453034779742</x:v>
+      </x:c>
+      <x:c r="J5" s="12" t="n">
+        <x:f>IFERROR(H5/F5,0)</x:f>
+        <x:v>0.2240453034779742</x:v>
+      </x:c>
+      <x:c r="K5" s="13" t="n">
+        <x:f>(I5-J5)*100</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L5" s="2" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="M5" s="2" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="N5" s="2" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="O5" s="2" t="str">
+        <x:f>IF(AND(C5=D5,E5=F5,G5=H5,L5="PASS",M5="PASS",OR(N5="PASS",N5="N/A")),"PASS","CHECK")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="34" customHeight="1">
+      <x:c r="A6" s="2" t="str">
+        <x:v>Los Angeles County</x:v>
+      </x:c>
+      <x:c r="B6" s="2" t="str">
+        <x:v>county=06037</x:v>
+      </x:c>
+      <x:c r="C6" s="11" t="n">
+        <x:v>223914</x:v>
+      </x:c>
+      <x:c r="D6" s="11" t="n">
+        <x:v>223914</x:v>
+      </x:c>
+      <x:c r="E6" s="11" t="n">
+        <x:v>152070</x:v>
+      </x:c>
+      <x:c r="F6" s="11" t="n">
+        <x:v>152070</x:v>
+      </x:c>
+      <x:c r="G6" s="11" t="n">
+        <x:v>36720</x:v>
+      </x:c>
+      <x:c r="H6" s="11" t="n">
+        <x:v>36720</x:v>
+      </x:c>
+      <x:c r="I6" s="12" t="n">
+        <x:f>IFERROR(G6/E6,0)</x:f>
+        <x:v>0.24146774511738014</x:v>
+      </x:c>
+      <x:c r="J6" s="12" t="n">
+        <x:f>IFERROR(H6/F6,0)</x:f>
+        <x:v>0.24146774511738014</x:v>
+      </x:c>
+      <x:c r="K6" s="13" t="n">
+        <x:f>(I6-J6)*100</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L6" s="2" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="M6" s="2" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="N6" s="2" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="O6" s="2" t="str">
+        <x:f>IF(AND(C6=D6,E6=F6,G6=H6,L6="PASS",M6="PASS",OR(N6="PASS",N6="N/A")),"PASS","CHECK")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="34" customHeight="1">
+      <x:c r="A7" s="2" t="str">
+        <x:v>California × conventional</x:v>
+      </x:c>
+      <x:c r="B7" s="2" t="str">
+        <x:v>state=CA; loan_type=1</x:v>
+      </x:c>
+      <x:c r="C7" s="11" t="n">
+        <x:v>961135</x:v>
+      </x:c>
+      <x:c r="D7" s="11" t="n">
+        <x:v>961135</x:v>
+      </x:c>
+      <x:c r="E7" s="11" t="n">
+        <x:v>670649</x:v>
+      </x:c>
+      <x:c r="F7" s="11" t="n">
+        <x:v>670649</x:v>
+      </x:c>
+      <x:c r="G7" s="11" t="n">
+        <x:v>153088</x:v>
+      </x:c>
+      <x:c r="H7" s="11" t="n">
+        <x:v>153088</x:v>
+      </x:c>
+      <x:c r="I7" s="12" t="n">
+        <x:f>IFERROR(G7/E7,0)</x:f>
+        <x:v>0.22826843848272346</x:v>
+      </x:c>
+      <x:c r="J7" s="12" t="n">
+        <x:f>IFERROR(H7/F7,0)</x:f>
+        <x:v>0.22826843848272346</x:v>
+      </x:c>
+      <x:c r="K7" s="13" t="n">
+        <x:f>(I7-J7)*100</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L7" s="2" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="M7" s="2" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="N7" s="2" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="O7" s="2" t="str">
+        <x:f>IF(AND(C7=D7,E7=F7,G7=H7,L7="PASS",M7="PASS",OR(N7="PASS",N7="N/A")),"PASS","CHECK")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="34" customHeight="1">
+      <x:c r="A8" s="2" t="str">
+        <x:v>Largest reporting institution (LEI)</x:v>
+      </x:c>
+      <x:c r="B8" s="2" t="str">
+        <x:v>one LEI selected by largest local 2025 action-1–8 count</x:v>
+      </x:c>
+      <x:c r="C8" s="11" t="n">
+        <x:v>663472</x:v>
+      </x:c>
+      <x:c r="D8" s="11" t="n">
+        <x:v>663472</x:v>
+      </x:c>
+      <x:c r="E8" s="11" t="n">
+        <x:v>555321</x:v>
+      </x:c>
+      <x:c r="F8" s="11" t="n">
+        <x:v>555321</x:v>
+      </x:c>
+      <x:c r="G8" s="11" t="n">
+        <x:v>110634</x:v>
+      </x:c>
+      <x:c r="H8" s="11" t="n">
+        <x:v>110634</x:v>
+      </x:c>
+      <x:c r="I8" s="12" t="n">
+        <x:f>IFERROR(G8/E8,0)</x:f>
+        <x:v>0.19922531292711784</x:v>
+      </x:c>
+      <x:c r="J8" s="12" t="n">
+        <x:f>IFERROR(H8/F8,0)</x:f>
+        <x:v>0.19922531292711784</x:v>
+      </x:c>
+      <x:c r="K8" s="13" t="n">
+        <x:f>(I8-J8)*100</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L8" s="2" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="M8" s="2" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="N8" s="2" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="O8" s="2" t="str">
+        <x:f>IF(AND(C8=D8,E8=F8,G8=H8,L8="PASS",M8="PASS",OR(N8="PASS",N8="N/A")),"PASS","CHECK")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="34" customHeight="1">
+      <x:c r="A9" s="2" t="str">
+        <x:v>Nationwide conventional loans</x:v>
+      </x:c>
+      <x:c r="B9" s="2" t="str">
+        <x:v>loan_type=1</x:v>
+      </x:c>
+      <x:c r="C9" s="11" t="n">
+        <x:v>10224134</x:v>
+      </x:c>
+      <x:c r="D9" s="11" t="n">
+        <x:v>10224134</x:v>
+      </x:c>
+      <x:c r="E9" s="11" t="n">
+        <x:v>7384608</x:v>
+      </x:c>
+      <x:c r="F9" s="11" t="n">
+        <x:v>7384608</x:v>
+      </x:c>
+      <x:c r="G9" s="11" t="n">
+        <x:v>1728114</x:v>
+      </x:c>
+      <x:c r="H9" s="11" t="n">
+        <x:v>1728114</x:v>
+      </x:c>
+      <x:c r="I9" s="12" t="n">
+        <x:f>IFERROR(G9/E9,0)</x:f>
+        <x:v>0.23401567151567151</x:v>
+      </x:c>
+      <x:c r="J9" s="12" t="n">
+        <x:f>IFERROR(H9/F9,0)</x:f>
+        <x:v>0.23401567151567151</x:v>
+      </x:c>
+      <x:c r="K9" s="13" t="n">
+        <x:f>(I9-J9)*100</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L9" s="2" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="M9" s="2" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="N9" s="2" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="O9" s="2" t="str">
+        <x:f>IF(AND(C9=D9,E9=F9,G9=H9,L9="PASS",M9="PASS",OR(N9="PASS",N9="N/A")),"PASS","CHECK")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="2"/>
+      <x:c r="B10" s="2"/>
+      <x:c r="C10" s="2"/>
+      <x:c r="D10" s="2"/>
+      <x:c r="E10" s="2"/>
+      <x:c r="F10" s="2"/>
+      <x:c r="G10" s="2"/>
+      <x:c r="H10" s="2"/>
+      <x:c r="I10" s="2"/>
+      <x:c r="J10" s="2"/>
+      <x:c r="K10" s="2"/>
+      <x:c r="L10" s="2"/>
+      <x:c r="M10" s="2"/>
+      <x:c r="N10" s="2"/>
+      <x:c r="O10" s="2"/>
+    </x:row>
+    <x:row r="11" ht="52" customHeight="1">
+      <x:c r="A11" s="7" t="str">
+        <x:v>Public sheet intentionally omits raw LAR rows, local paths, exact LEI and full action-level query responses. Exact query, LEI, action profiles, API payloads and receipt hashes are retained in the private D: receipt; only aggregate summaries are published.</x:v>
+      </x:c>
+      <x:c r="B11" s="7"/>
+      <x:c r="C11" s="7"/>
+      <x:c r="D11" s="7"/>
+      <x:c r="E11" s="7"/>
+      <x:c r="F11" s="7"/>
+      <x:c r="G11" s="7"/>
+      <x:c r="H11" s="7"/>
+      <x:c r="I11" s="7"/>
+      <x:c r="J11" s="7"/>
+      <x:c r="K11" s="7"/>
+      <x:c r="L11" s="7"/>
+      <x:c r="M11" s="7"/>
+      <x:c r="N11" s="7"/>
+      <x:c r="O11" s="7"/>
+    </x:row>
+    <x:row r="12" ht="52" customHeight="1">
+      <x:c r="A12" s="7"/>
+      <x:c r="B12" s="7"/>
+      <x:c r="C12" s="7"/>
+      <x:c r="D12" s="7"/>
+      <x:c r="E12" s="7"/>
+      <x:c r="F12" s="7"/>
+      <x:c r="G12" s="7"/>
+      <x:c r="H12" s="7"/>
+      <x:c r="I12" s="7"/>
+      <x:c r="J12" s="7"/>
+      <x:c r="K12" s="7"/>
+      <x:c r="L12" s="7"/>
+      <x:c r="M12" s="7"/>
+      <x:c r="N12" s="7"/>
+      <x:c r="O12" s="7"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="2"/>
+      <x:c r="B13" s="2"/>
+      <x:c r="C13" s="2"/>
+      <x:c r="D13" s="2"/>
+      <x:c r="E13" s="2"/>
+      <x:c r="F13" s="2"/>
+      <x:c r="G13" s="2"/>
+      <x:c r="H13" s="2"/>
+      <x:c r="I13" s="2"/>
+      <x:c r="J13" s="2"/>
+      <x:c r="K13" s="2"/>
+      <x:c r="L13" s="2"/>
+      <x:c r="M13" s="2"/>
+      <x:c r="N13" s="2"/>
+      <x:c r="O13" s="2"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="2"/>
+      <x:c r="B14" s="2"/>
+      <x:c r="C14" s="2"/>
+      <x:c r="D14" s="2"/>
+      <x:c r="E14" s="2"/>
+      <x:c r="F14" s="2"/>
+      <x:c r="G14" s="2"/>
+      <x:c r="H14" s="2"/>
+      <x:c r="I14" s="2"/>
+      <x:c r="J14" s="2"/>
+      <x:c r="K14" s="2"/>
+      <x:c r="L14" s="2"/>
+      <x:c r="M14" s="2"/>
+      <x:c r="N14" s="2"/>
+      <x:c r="O14" s="2"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="2"/>
+      <x:c r="B15" s="2"/>
+      <x:c r="C15" s="2"/>
+      <x:c r="D15" s="2"/>
+      <x:c r="E15" s="2"/>
+      <x:c r="F15" s="2"/>
+      <x:c r="G15" s="2"/>
+      <x:c r="H15" s="2"/>
+      <x:c r="I15" s="2"/>
+      <x:c r="J15" s="2"/>
+      <x:c r="K15" s="2"/>
+      <x:c r="L15" s="2"/>
+      <x:c r="M15" s="2"/>
+      <x:c r="N15" s="2"/>
+      <x:c r="O15" s="2"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="2"/>
+      <x:c r="B16" s="2"/>
+      <x:c r="C16" s="2"/>
+      <x:c r="D16" s="2"/>
+      <x:c r="E16" s="2"/>
+      <x:c r="F16" s="2"/>
+      <x:c r="G16" s="2"/>
+      <x:c r="H16" s="2"/>
+      <x:c r="I16" s="2"/>
+      <x:c r="J16" s="2"/>
+      <x:c r="K16" s="2"/>
+      <x:c r="L16" s="2"/>
+      <x:c r="M16" s="2"/>
+      <x:c r="N16" s="2"/>
+      <x:c r="O16" s="2"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="2"/>
+      <x:c r="B17" s="2"/>
+      <x:c r="C17" s="2"/>
+      <x:c r="D17" s="2"/>
+      <x:c r="E17" s="2"/>
+      <x:c r="F17" s="2"/>
+      <x:c r="G17" s="2"/>
+      <x:c r="H17" s="2"/>
+      <x:c r="I17" s="2"/>
+      <x:c r="J17" s="2"/>
+      <x:c r="K17" s="2"/>
+      <x:c r="L17" s="2"/>
+      <x:c r="M17" s="2"/>
+      <x:c r="N17" s="2"/>
+      <x:c r="O17" s="2"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="2"/>
+      <x:c r="B18" s="2"/>
+      <x:c r="C18" s="2"/>
+      <x:c r="D18" s="2"/>
+      <x:c r="E18" s="2"/>
+      <x:c r="F18" s="2"/>
+      <x:c r="G18" s="2"/>
+      <x:c r="H18" s="2"/>
+      <x:c r="I18" s="2"/>
+      <x:c r="J18" s="2"/>
+      <x:c r="K18" s="2"/>
+      <x:c r="L18" s="2"/>
+      <x:c r="M18" s="2"/>
+      <x:c r="N18" s="2"/>
+      <x:c r="O18" s="2"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="2"/>
+      <x:c r="B19" s="2"/>
+      <x:c r="C19" s="2"/>
+      <x:c r="D19" s="2"/>
+      <x:c r="E19" s="2"/>
+      <x:c r="F19" s="2"/>
+      <x:c r="G19" s="2"/>
+      <x:c r="H19" s="2"/>
+      <x:c r="I19" s="2"/>
+      <x:c r="J19" s="2"/>
+      <x:c r="K19" s="2"/>
+      <x:c r="L19" s="2"/>
+      <x:c r="M19" s="2"/>
+      <x:c r="N19" s="2"/>
+      <x:c r="O19" s="2"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="2"/>
+      <x:c r="B20" s="2"/>
+      <x:c r="C20" s="2"/>
+      <x:c r="D20" s="2"/>
+      <x:c r="E20" s="2"/>
+      <x:c r="F20" s="2"/>
+      <x:c r="G20" s="2"/>
+      <x:c r="H20" s="2"/>
+      <x:c r="I20" s="2"/>
+      <x:c r="J20" s="2"/>
+      <x:c r="K20" s="2"/>
+      <x:c r="L20" s="2"/>
+      <x:c r="M20" s="2"/>
+      <x:c r="N20" s="2"/>
+      <x:c r="O20" s="2"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:O1"/>
+    <x:mergeCell ref="A2:O2"/>
+    <x:mergeCell ref="A11:O12"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4605d0f6e68495e"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -2671,12 +3275,12 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf4274708d8b4302"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5a2883a83264d5a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -2828,93 +3432,101 @@
     </x:row>
     <x:row r="12" ht="52" customHeight="1">
       <x:c r="A12" s="14" t="str">
-        <x:v>2025 Dynamic</x:v>
+        <x:v>2025 filtered API dimension check</x:v>
       </x:c>
       <x:c r="B12" s="14" t="str">
-        <x:v>Dynamic is a separate weekly release state; not the Browser-selected static Snapshot.</x:v>
+        <x:v>5 Snapshot scopes reconciled; four app marginal buckets match and the California × loan-type intersection is raw/API-only.</x:v>
       </x:c>
       <x:c r="C12" s="14" t="str">
-        <x:v>2025 Snapshot/Dynamic comparison report</x:v>
+        <x:v>See Dimension parity and sanitized API audit JSON</x:v>
       </x:c>
       <x:c r="D12" s="14" t="str">
-        <x:v>Separate source ID</x:v>
+        <x:v>PASS</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="52" customHeight="1">
       <x:c r="A13" s="14" t="str">
-        <x:v>Release-state limits</x:v>
+        <x:v>2025 Dynamic</x:v>
       </x:c>
       <x:c r="B13" s="14" t="str">
-        <x:v>Release differences can include late submissions/resubmissions and reclassifications; action deltas can have either sign.</x:v>
+        <x:v>Dynamic is a separate weekly release state; not the Browser-selected static Snapshot.</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>No row matching performed</x:v>
+        <x:v>2025 Snapshot/Dynamic comparison report</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
-        <x:v>Do not call new unique rows</x:v>
+        <x:v>Separate source ID</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="52" customHeight="1">
       <x:c r="A14" s="14" t="str">
-        <x:v>Trend limits</x:v>
+        <x:v>Release-state limits</x:v>
       </x:c>
       <x:c r="B14" s="14" t="str">
-        <x:v>Across-year levels also reflect coverage, reporting thresholds, product mix and geography mix.</x:v>
+        <x:v>Release differences can include late submissions/resubmissions and reclassifications; action deltas can have either sign.</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
-        <x:v>Additional harmonization needed</x:v>
+        <x:v>No row matching performed</x:v>
       </x:c>
       <x:c r="D14" s="14" t="str">
-        <x:v>Not causal</x:v>
+        <x:v>Do not call new unique rows</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="52" customHeight="1">
       <x:c r="A15" s="14" t="str">
-        <x:v>Data handling</x:v>
+        <x:v>Trend limits</x:v>
       </x:c>
       <x:c r="B15" s="14" t="str">
-        <x:v>This workbook has action-count aggregates, no raw LAR records. Raw CSV/ZIP and full source receipts remain private.</x:v>
+        <x:v>Across-year levels also reflect coverage, reporting thresholds, product mix and geography mix.</x:v>
       </x:c>
       <x:c r="C15" s="14" t="str">
-        <x:v>Project rights review</x:v>
+        <x:v>Additional harmonization needed</x:v>
       </x:c>
       <x:c r="D15" s="14" t="str">
-        <x:v>No row-level data</x:v>
+        <x:v>Not causal</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="52" customHeight="1">
       <x:c r="A16" s="14" t="str">
-        <x:v>Rights status</x:v>
+        <x:v>Data handling</x:v>
       </x:c>
       <x:c r="B16" s="14" t="str">
-        <x:v>Reviewed pages support analysis/privacy-modified use but did not specify raw rehosting/redistribution terms.</x:v>
+        <x:v>This workbook has action-count aggregates, no raw LAR records. Raw CSV/ZIP and full source receipts remain private.</x:v>
       </x:c>
       <x:c r="C16" s="14" t="str">
-        <x:v>HMDA rights review</x:v>
+        <x:v>Project rights review</x:v>
       </x:c>
       <x:c r="D16" s="14" t="str">
-        <x:v>Raw remains private</x:v>
+        <x:v>No row-level data</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="52" customHeight="1">
       <x:c r="A17" s="14" t="str">
+        <x:v>Rights status</x:v>
+      </x:c>
+      <x:c r="B17" s="14" t="str">
+        <x:v>Reviewed pages support analysis/privacy-modified use but did not specify raw rehosting/redistribution terms.</x:v>
+      </x:c>
+      <x:c r="C17" s="14" t="str">
+        <x:v>HMDA rights review</x:v>
+      </x:c>
+      <x:c r="D17" s="14" t="str">
+        <x:v>Raw remains private</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="52" customHeight="1">
+      <x:c r="A18" s="14" t="str">
         <x:v>Forecast/model</x:v>
       </x:c>
-      <x:c r="B17" s="14" t="str">
+      <x:c r="B18" s="14" t="str">
         <x:v>No forecast, imputation, PD, default or risk model was created by this audit.</x:v>
       </x:c>
-      <x:c r="C17" s="14" t="str">
+      <x:c r="C18" s="14" t="str">
         <x:v>Audit scope</x:v>
       </x:c>
-      <x:c r="D17" s="14" t="str">
+      <x:c r="D18" s="14" t="str">
         <x:v>None</x:v>
       </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="2"/>
-      <x:c r="B18" s="2"/>
-      <x:c r="C18" s="2"/>
-      <x:c r="D18" s="2"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="2"/>
@@ -2982,7 +3594,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd72bd63cba13402b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23c402b0cd374728"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add receipt-verified HMDA intersection filters
</commit_message>
<xml_diff>
--- a/apps/excel/templates/CreditAtlas-HMDA-Browser-Release-Audit-2018-2025.xlsx
+++ b/apps/excel/templates/CreditAtlas-HMDA-Browser-Release-Audit-2018-2025.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Browser selected" sheetId="1" r:id="Re5f2c24140564ba5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App One-Year" sheetId="2" r:id="Ra40549d9b13b435a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vintage deltas" sheetId="3" r:id="Rf103529d0f314adc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dimension parity" sheetId="4" r:id="Rd0ddb561d3ca46ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lineage" sheetId="5" r:id="R58fb6add88fb4e67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method &amp; sources" sheetId="6" r:id="R9a99abe7817e428b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Browser selected" sheetId="1" r:id="R701142bae61545b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App One-Year" sheetId="2" r:id="Rdfed85791ce54df7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vintage deltas" sheetId="3" r:id="Re9e7041285db4b4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dimension parity" sheetId="4" r:id="R2dcef0d3b8d34515"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lineage" sheetId="5" r:id="R9e7f38d2a4e74ec5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method &amp; sources" sheetId="6" r:id="R7b7007d315ed4d95"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -216,7 +216,7 @@
     <x:tableColumn id="11" name="Δ share · pp"/>
     <x:tableColumn id="12" name="Local raw match"/>
     <x:tableColumn id="13" name="API filter echo"/>
-    <x:tableColumn id="14" name="App marginal match"/>
+    <x:tableColumn id="14" name="App match"/>
     <x:tableColumn id="15" name="Check"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1118,7 +1118,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a6dbaa99e70428e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11c0d32b46d44e48"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1732,7 +1732,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re89fe6e681e44e8e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref2e9525ca454af9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2378,7 +2378,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ad22e8bbef94eb5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc96c48d796aa4602"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2425,7 +2425,7 @@
     </x:row>
     <x:row r="2" ht="54" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Five spot-check scopes compared on action codes 1–8. Four marginal scopes also match the receipt-verified app report; California × product is raw/API validated but not an app intersection. Share columns are Excel formulas.</x:v>
+        <x:v>Five spot-check scopes compared on action codes 1–8. Four app marginal buckets and the California × conventional intersection match the receipt-verified app report. Share columns are Excel formulas.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -2500,7 +2500,7 @@
         <x:v>API filter echo</x:v>
       </x:c>
       <x:c r="N4" s="10" t="str">
-        <x:v>App marginal match</x:v>
+        <x:v>App match</x:v>
       </x:c>
       <x:c r="O4" s="10" t="str">
         <x:v>Check</x:v>
@@ -2652,7 +2652,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="N7" s="2" t="str">
-        <x:v>N/A</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="O7" s="2" t="str">
         <x:f>IF(AND(C7=D7,E7=F7,G7=H7,L7="PASS",M7="PASS",OR(N7="PASS",N7="N/A")),"PASS","CHECK")</x:f>
@@ -2958,7 +2958,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4605d0f6e68495e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R639b255c9c404873"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3275,7 +3275,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5a2883a83264d5a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffcc02ed47164543"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3435,7 +3435,7 @@
         <x:v>2025 filtered API dimension check</x:v>
       </x:c>
       <x:c r="B12" s="14" t="str">
-        <x:v>5 Snapshot scopes reconciled; four app marginal buckets match and the California × loan-type intersection is raw/API-only.</x:v>
+        <x:v>5 Snapshot scopes reconciled; four app marginal buckets and the California × conventional intersection match.</x:v>
       </x:c>
       <x:c r="C12" s="14" t="str">
         <x:v>See Dimension parity and sanitized API audit JSON</x:v>
@@ -3594,7 +3594,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23c402b0cd374728"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6496fd65fac4eaf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>